<commit_message>
Add guidance notes to parameter template headers
</commit_message>
<xml_diff>
--- a/templates/Template_Consulta_Parametros_Revit_IFC.xlsx
+++ b/templates/Template_Consulta_Parametros_Revit_IFC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\0000_pset_compo\Information-Manager-IFC-skill\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3BF3B45F-4D62-4745-9633-B7EC691C9D26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B38556C-2A79-488E-8B74-72D2F4A077D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CC375436-FAE1-4126-B745-F1DE9183DA82}"/>
   </bookViews>
@@ -41,6 +41,1466 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Jeff Lima</author>
+  </authors>
+  <commentList>
+    <comment ref="A5" authorId="0" shapeId="0" xr:uid="{D72ABF14-D72D-4E15-A43F-8C7EB0D53DFF}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Identificador único e estável do requisito. Ex.: ARQ-PORTA-001. Deve permanecer igual em todos os gates.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B5" authorId="0" shapeId="0" xr:uid="{8DCA41F4-F6D3-4782-99CA-1871CD297456}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Descrição original do dado solicitado pelo cliente, sem reinterpretar silenciosamente.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C5" authorId="0" shapeId="0" xr:uid="{054119E2-3082-47CB-A5A1-BF8689550132}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Decisão, uso BIM ou processo que justifica a necessidade da informação.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0" xr:uid="{03D617BD-0E4D-44A1-B65B-AE2BBDD7E5E9}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Disciplina responsável ou à qual o requisito se aplica. Ex.: Arquitetura, Estrutura.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E5" authorId="0" shapeId="0" xr:uid="{97AC1022-B243-44AF-9948-DB084DD23BAB}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Categoria autoral do Revit à qual o requisito se aplica. Ex.: Doors, Walls, Floors.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F5" authorId="0" shapeId="0" xr:uid="{EFBDE662-BA32-4D23-9E07-1EDE2120131C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Família ou tipo usado como referência para avaliar o requisito. Não torna o requisito exclusivo desse exemplo.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G5" authorId="0" shapeId="0" xr:uid="{3818407D-0709-48D5-8E87-978AC8A34826}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Indica onde o dado vive no Revit: instance, type ou unspecified.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H5" authorId="0" shapeId="0" xr:uid="{645D1314-194C-4089-AE8E-A1DAF527D04E}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Unidade da grandeza. Ex.: mm, m², m³. Use N/A para textos, booleanos ou identificadores.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I5" authorId="0" shapeId="0" xr:uid="{A796D50C-A9AE-4B85-A719-7EB2232A961F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Natureza esperada do valor: text, integer, real, boolean, length, area, volume, identifier, date etc.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J5" authorId="0" shapeId="0" xr:uid="{2AD19DC1-789F-4EAF-A820-955E7A9320FA}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Quantidade mínima e máxima de valores admitidos. 0..1 = opcional e único; 1 = obrigatório e único; 0..n = opcional e repetível; 1..n = pelo menos um. Orienta a cardinalidade do IDS.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K5" authorId="0" shapeId="0" xr:uid="{B60CC5C2-1BB2-45B1-A72D-5D9164297221}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Lista, faixa, padrão ou enumeração admitida. Ex.: 30; 60; 90 ou Sim/Não. Deixe vazio quando livre.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L5" authorId="0" shapeId="0" xr:uid="{ACB1B6F7-4A34-4EDD-BD52-28B14C72AC5C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Fase em que o dado se torna obrigatório. Ex.: Projeto executivo, Construção ou Operação.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M5" authorId="0" shapeId="0" xr:uid="{2289FD41-CA09-40CB-8DB8-D80FEC760B62}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Versão exata do schema de entrega: IFC2X3, IFC4 ou IFC4.3. Não misture templates entre schemas.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N5" authorId="0" shapeId="0" xr:uid="{7F990084-1255-4129-BE99-D7AFCFF80F04}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Classe IFC inicialmente considerada para o objeto. É candidata até a validação técnica.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O5" authorId="0" shapeId="0" xr:uid="{9A8B6886-EDED-49C9-ACA5-19232D0806BE}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+PredefinedType inicialmente considerado. Preencher somente quando existir e for aplicável no schema.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="P5" authorId="0" shapeId="0" xr:uid="{61906A94-9BEE-4480-91E0-9E55600A648C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Pset inicialmente considerado. É apenas candidato; não combine automaticamente Pset e Qto.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Q5" authorId="0" shapeId="0" xr:uid="{755A232A-D378-4ECA-BC70-377FC2689830}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Nome da propriedade IFC inicialmente considerada dentro do Pset candidato.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="R5" authorId="0" shapeId="0" xr:uid="{B0679FEB-6BAC-40A2-870F-A76F2D73B04E}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Regra objetiva de aprovação. Deve permitir que outra pessoa chegue à mesma decisão.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="S5" authorId="0" shapeId="0" xr:uid="{14E95F32-2DEF-4430-9FE4-2ED2AD84D25E}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Documento, planilha, aba, linha ou identificador do requisito recebido do cliente.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="T5" authorId="0" shapeId="0" xr:uid="{764863F8-C16C-4CD8-8287-6AC55E1DBBF7}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Contexto adicional, dúvidas, exceções ou premissas. Não usar para esconder requisito indefinido.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Jeff Lima</author>
+  </authors>
+  <commentList>
+    <comment ref="A5" authorId="0" shapeId="0" xr:uid="{DFBE62A1-9492-49EF-A7CE-E3FFF55EE7A4}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Mesmo identificador estável recebido na entrada.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B5" authorId="0" shapeId="0" xr:uid="{652446EE-36F1-4415-8506-3A8B56F04573}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Descrição interpretada e normalizada, preservando o sentido aprovado do requisito.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C5" authorId="0" shapeId="0" xr:uid="{C68CFAA3-F5D4-42C1-8B30-B12412C112F5}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Classificação da origem/autoria: NATIVO_REVIT, NATIVO_IFC, PARAMETRO_COMPARTILHADO, CALCULADO, CONFLITO etc.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0" xr:uid="{827D06CB-AE5B-492F-8779-63F29CBFCC55}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Ação aprovada: CREATE, REUSE, MAP, CALCULATE, REMOVE_DUPLICATE, NO_ACTION ou REVIEW.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E5" authorId="0" shapeId="0" xr:uid="{684217F6-E1A1-4B79-B0CB-6128E8493CDA}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Motivo técnico da classificação e da ação, apoiado por evidência.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F5" authorId="0" shapeId="0" xr:uid="{FCC2E5BD-0C71-4DCE-9D17-9B42C3FBB2F9}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Nome exato do parâmetro autoral no Revit.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G5" authorId="0" shapeId="0" xr:uid="{52644D09-E047-4BFF-A0AB-6425CCF81214}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Escopo real do parâmetro: instance, type ou unspecified.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H5" authorId="0" shapeId="0" xr:uid="{7D3FDF74-CAE5-4DE8-B621-4E1B1BF7D804}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Tipo de dado no Revit. Deve ser compatível com a unidade e o datatype IFC.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I5" authorId="0" shapeId="0" xr:uid="{A4EDDD23-A302-44AB-9653-C00AF280EE94}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Categorias Revit vinculadas ao parâmetro. Separar múltiplas categorias de forma consistente.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J5" authorId="0" shapeId="0" xr:uid="{7EA2E6EE-C952-4F75-825F-F3FC90F9EBF5}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+GUID controlado do parâmetro compartilhado. Use PENDING até aprovação; não invente GUID.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K5" authorId="0" shapeId="0" xr:uid="{0A79CE12-BEF0-4237-947D-FE9414844379}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Grupo de parâmetros do Revit usado para organização da interface.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L5" authorId="0" shapeId="0" xr:uid="{61C4BC4D-8B26-425A-8F3A-0B1AD0A6985C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Schema IFC exato usado na decisão e na exportação.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M5" authorId="0" shapeId="0" xr:uid="{3017A73B-E54F-4428-BBE3-59C2295461D1}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Classe IFC final aprovada e posteriormente comprovada no arquivo exportado.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N5" authorId="0" shapeId="0" xr:uid="{969D7B43-7A0A-448C-AF61-05DCE5DAC057}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+PredefinedType final. Preencher somente quando aplicável e comprovado.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O5" authorId="0" shapeId="0" xr:uid="{7A837C29-4650-4A12-B6B9-590BB037652D}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Destino técnico: ATTRIBUTE, STANDARD_QTO, CUSTOM_QTO, STANDARD_PSET, CUSTOM_PSET, MATERIAL_ASSOCIATION, CALCULATED_ONLY ou UNVERIFIED.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="P5" authorId="0" shapeId="0" xr:uid="{1B2C0ABD-FFFB-46C6-93B2-2C134287FA5C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Atributo nativo IFC. Ex.: IfcDoor.OverallWidth. Preencher somente quando Destino_IFC_Tipo = ATTRIBUTE.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Q5" authorId="0" shapeId="0" xr:uid="{EEA6D534-4ED1-4AD1-A351-316794F7D133}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Nome do conjunto de quantidades. Validar no schema exato; não transportar nomes entre IFC2X3 e IFC4/4.3.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="R5" authorId="0" shapeId="0" xr:uid="{738A4D32-2A6E-4D7A-95FE-E1D191C0A7FB}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Nome da quantidade dentro do QuantitySet. Ex.: GrossArea, Length ou NetVolume.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="S5" authorId="0" shapeId="0" xr:uid="{8867D81C-9CC3-4D6E-84B0-C380DFCA0BA5}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Subtipo IFC da quantidade. Ex.: IfcQuantityLength, IfcQuantityArea ou IfcQuantityVolume.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="T5" authorId="0" shapeId="0" xr:uid="{141CB259-9571-48F0-94F3-C7D58FD9AA17}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Método de medição que define como a quantidade foi obtida. Essencial para comparar valores de forma consistente.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="U5" authorId="0" shapeId="0" xr:uid="{2671853F-EA03-4D86-93DD-6D01594CFC24}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Fórmula ou regra reproduzível do cálculo, incluindo entradas e tratamento de exceções.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="V5" authorId="0" shapeId="0" xr:uid="{286AC176-4598-4777-B06B-B8FF42F4F1F8}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Nome do Property Set. Preencher apenas para STANDARD_PSET ou CUSTOM_PSET.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="W5" authorId="0" shapeId="0" xr:uid="{61426EA6-A248-4282-8A6E-66B7EE198FC5}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Nome da propriedade dentro do Pset.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="X5" authorId="0" shapeId="0" xr:uid="{EF051856-5F8B-4306-BEA4-731E0885EF2C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Datatype IFC final. Ex.: IfcLabel, IfcIdentifier, IfcLengthMeasure ou IfcAreaMeasure.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Y5" authorId="0" shapeId="0" xr:uid="{0A42C329-0815-4109-B681-09CEBB425131}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Associação IFC usada para material. Preferir associação semântica ao texto duplicado quando representar material efetivo.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Z5" authorId="0" shapeId="0" xr:uid="{2EF95991-321E-479C-BE23-75326490CA5B}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Como Revit/exportador transforma a origem no destino IFC.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AA5" authorId="0" shapeId="0" xr:uid="{497E2E75-BFE4-475E-981E-268D720C1332}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Fonte real do valor: parâmetro nativo, geometria, cálculo, parâmetro compartilhado ou fonte externa aprovada.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AB5" authorId="0" shapeId="0" xr:uid="{3B9D527A-1301-4B1C-9A11-EF0C4A7B4238}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Tipo da fonte consultada. Ex.: revit-shared, user-defined-pset, schema-ifc ou cobie-ifc2x3.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AC5" authorId="0" shapeId="0" xr:uid="{4BC9C2E2-F61F-4C0D-B6D1-78AA342B0F3F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Arquivo, URI ou conjunto aprovado que sustenta a decisão.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AD5" authorId="0" shapeId="0" xr:uid="{678A2360-2410-4C32-AE96-7235B3F2BA7D}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Linha ou posição precisa dentro do arquivo-fonte, quando aplicável.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AE5" authorId="0" shapeId="0" xr:uid="{57772EEE-45C1-4BB9-A7C9-22290D8818D0}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Entidade realmente encontrada no IFC. Ex.: IfcPropertySingleValue, IfcElementQuantity ou IfcQuantityArea.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AF5" authorId="0" shapeId="0" xr:uid="{F6B99869-509C-421F-BE6B-379068C07F40}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Evidência objetiva da inspeção: arquivo/hash, GlobalId, caminho da entidade, valor e ferramenta.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AG5" authorId="0" shapeId="0" xr:uid="{886DD81F-1C1F-4BC9-9BF7-5F248DBE4D07}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Indica conflito de nome, GUID, datatype, unidade, escopo, categoria ou destino.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AH5" authorId="0" shapeId="0" xr:uid="{B5BF982E-4797-40D2-AF28-47069406FEC9}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Restrições conhecidas da decisão ou da ferramenta. Limitação relevante impede aprovação silenciosa.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AI5" authorId="0" shapeId="0" xr:uid="{1756D16A-6444-42AC-88ED-4530A173401F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Sim quando a decisão exige validação semântica, exceção, criação, publicação ou mudança no modelo.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AJ5" authorId="0" shapeId="0" xr:uid="{595F23F2-A814-468B-BED3-8B81C92936CA}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Função ou pessoa responsável pela aprovação. Evitar dado pessoal desnecessário; preferir papel.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AK5" authorId="0" shapeId="0" xr:uid="{FDE19079-F3BE-4ABE-B73B-38F358B32549}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Estado da decisão: RASCUNHO, EM_REVISAO, APROVADO, REPROVADO ou REVISAO_HUMANA.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AL5" authorId="0" shapeId="0" xr:uid="{E7B6A816-3C33-4323-A5B8-74859A57A6EC}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Versão controlada da matriz/regra que produziu o resultado.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AM5" authorId="0" shapeId="0" xr:uid="{7AEBF326-41BB-43D9-BBEB-BE0C659352FE}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Data da análise no formato de data do Excel, não como texto livre.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AN5" authorId="0" shapeId="0" xr:uid="{2DE723A6-6EBE-4E31-BFEC-3257C0E861EB}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Jeff Lima:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Notas finais, exceções e próximos passos que não cabem nos campos estruturados.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="231">
   <si>
@@ -741,7 +2201,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -785,6 +2245,19 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -2080,6 +3553,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2498,7 +3975,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54296401-7BB5-4C16-95CB-A0A7BED3DEA2}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54296401-7BB5-4C16-95CB-A0A7BED3DEA2}">
   <dimension ref="A1:T8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2832,8 +4309,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <legacyDrawing r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -2881,7 +4359,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4FDE0B4-DF20-4BFB-8CA7-E1E3C1BF7F01}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4FDE0B4-DF20-4BFB-8CA7-E1E3C1BF7F01}">
   <sheetPr>
     <tabColor rgb="FF2E74B5"/>
   </sheetPr>
@@ -2890,7 +4368,7 @@
   <cols>
     <col min="1" max="1" width="76.7109375" customWidth="1"/>
     <col min="2" max="2" width="30.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="28.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.85546875" customWidth="1"/>
     <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="61.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="27.140625" bestFit="1" customWidth="1"/>
@@ -3476,8 +4954,9 @@
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <legacyDrawing r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">

</xml_diff>

<commit_message>
Update PIR EIR guidance and parameter template
</commit_message>
<xml_diff>
--- a/templates/Template_Consulta_Parametros_Revit_IFC.xlsx
+++ b/templates/Template_Consulta_Parametros_Revit_IFC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\0000_pset_compo\Information-Manager-IFC-skill\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B38556C-2A79-488E-8B74-72D2F4A077D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BA41DF2-844A-43F6-8E0F-C6265B6052DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CC375436-FAE1-4126-B745-F1DE9183DA82}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{CC375436-FAE1-4126-B745-F1DE9183DA82}"/>
   </bookViews>
   <sheets>
     <sheet name="Entrada_Requisitos" sheetId="1" r:id="rId1"/>
@@ -57,6 +57,286 @@
             <rFont val="Segoe UI"/>
             <family val="2"/>
           </rPr>
+          <t>Identificador único e estável do requisito. Não é o nome do parâmetro.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B5" authorId="0" shapeId="0" xr:uid="{8DCA41F4-F6D3-4782-99CA-1871CD297456}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Nome do campo conforme recebido do cliente, preservado para rastreabilidade.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C5" authorId="0" shapeId="0" xr:uid="{054119E2-3082-47CB-A5A1-BF8689550132}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Descrição clara do conteúdo informacional exigido.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="D5" authorId="0" shapeId="0" xr:uid="{03D617BD-0E4D-44A1-B65B-AE2BBDD7E5E9}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Uso ou decisão que justifica a coleta e validação deste dado.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="E5" authorId="0" shapeId="0" xr:uid="{97AC1022-B243-44AF-9948-DB084DD23BAB}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Disciplina responsável pelo requisito e pela correção do modelo.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F5" authorId="0" shapeId="0" xr:uid="{EFBDE662-BA32-4D23-9E07-1EDE2120131C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Categoria do Revit na qual o parâmetro deve ser investigado.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G5" authorId="0" shapeId="0" xr:uid="{3818407D-0709-48D5-8E87-978AC8A34826}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Família ou tipo de referência, quando o requisito não se aplica à categoria inteira.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H5" authorId="0" shapeId="0" xr:uid="{645D1314-194C-4089-AE8E-A1DAF527D04E}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Nome provável do parâmetro no Revit. Deve ser confirmado como nativo, compartilhado, de projeto ou inexistente.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="I5" authorId="0" shapeId="0" xr:uid="{A796D50C-A9AE-4B85-A719-7EB2232A961F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Origem técnica do dado no Revit: NATIVO, COMPARTILHADO, PROJETO, CALCULADO, CONFIGURACAO_EXPORTACAO, INEXISTENTE, EXTERNO ou UNVERIFIED.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="J5" authorId="0" shapeId="0" xr:uid="{2AD19DC1-789F-4EAF-A820-955E7A9320FA}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Indica se o valor pertence à instância ou ao tipo no Revit.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="K5" authorId="0" shapeId="0" xr:uid="{B60CC5C2-1BB2-45B1-A72D-5D9164297221}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Unidade esperada, por exemplo mm, m, m², m³, kg ou sem unidade.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L5" authorId="0" shapeId="0" xr:uid="{ACB1B6F7-4A34-4EDD-BD52-28B14C72AC5C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Tipo lógico esperado: texto, número, comprimento, área, volume, booleano, enumeração etc.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="M5" authorId="0" shapeId="0" xr:uid="{2289FD41-CA09-40CB-8DB8-D80FEC760B62}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Quantidade mínima e máxima de ocorrências do dado. Exemplos: 1, 0..1 e 1..n.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N5" authorId="0" shapeId="0" xr:uid="{7F990084-1255-4129-BE99-D7AFCFF80F04}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Lista controlada de valores aceitos, quando aplicável.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="O5" authorId="0" shapeId="0" xr:uid="{9A8B6886-EDED-49C9-ACA5-19232D0806BE}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Etapa em que o requisito passa a ser obrigatório.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="P5" authorId="0" shapeId="0" xr:uid="{61906A94-9BEE-4480-91E0-9E55600A648C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Versão IFC contratada para análise, como IFC2X3 ou IFC4.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Q5" authorId="0" shapeId="0" xr:uid="{755A232A-D378-4ECA-BC70-377FC2689830}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Classe IFC provável do objeto. Deve ser confirmada contra o schema contratado.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="R5" authorId="0" shapeId="0" xr:uid="{B0679FEB-6BAC-40A2-870F-A76F2D73B04E}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>PredefinedType aplicável, quando necessário para delimitar a população.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="S5" authorId="0" shapeId="0" xr:uid="{14E95F32-2DEF-4430-9FE4-2ED2AD84D25E}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Natureza do destino IFC candidato: ATTRIBUTE, STANDARD_QTO, CUSTOM_QTO, STANDARD_PSET, CUSTOM_PSET ou UNVERIFIED.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="T5" authorId="0" shapeId="0" xr:uid="{764863F8-C16C-4CD8-8287-6AC55E1DBBF7}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <family val="2"/>
+          </rPr>
+          <t>Atributo direto da entidade IFC, por exemplo Name, Description ou ObjectType. Não começa com Pset_.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="U5" authorId="0" shapeId="0" xr:uid="{04F2C6A0-8F26-4F74-80AD-6D3C1A27BF94}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <charset val="1"/>
+          </rPr>
           <t>Jeff Lima:</t>
         </r>
         <r>
@@ -64,22 +344,22 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Segoe UI"/>
-            <family val="2"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
-Identificador único e estável do requisito. Ex.: ARQ-PORTA-001. Deve permanecer igual em todos os gates.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="B5" authorId="0" shapeId="0" xr:uid="{8DCA41F4-F6D3-4782-99CA-1871CD297456}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
+Nome do conjunto de quantidades candidato, normalmente iniciado por Qto_ quando padronizado.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="V5" authorId="0" shapeId="0" xr:uid="{AAA2A283-2B61-416A-9218-19A18E2C7A3A}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <charset val="1"/>
           </rPr>
           <t>Jeff Lima:</t>
         </r>
@@ -88,22 +368,22 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Segoe UI"/>
-            <family val="2"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
-Descrição original do dado solicitado pelo cliente, sem reinterpretar silenciosamente.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C5" authorId="0" shapeId="0" xr:uid="{054119E2-3082-47CB-A5A1-BF8689550132}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
+Nome da quantidade dentro do QuantitySet, por exemplo GrossArea, NetVolume, Width ou Height.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="W5" authorId="0" shapeId="0" xr:uid="{48E7D5F4-0F11-4CB0-849C-B0B87A2EFE48}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <charset val="1"/>
           </rPr>
           <t>Jeff Lima:</t>
         </r>
@@ -112,22 +392,22 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Segoe UI"/>
-            <family val="2"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
-Decisão, uso BIM ou processo que justifica a necessidade da informação.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="D5" authorId="0" shapeId="0" xr:uid="{03D617BD-0E4D-44A1-B65B-AE2BBDD7E5E9}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
+Nome do Property Set candidato. Use Pset_ apenas para conjunto padronizado; conjunto próprio deve seguir governança do projeto.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="X5" authorId="0" shapeId="0" xr:uid="{6BA0A31C-93C0-4264-AF62-BC8880B1A381}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <charset val="1"/>
           </rPr>
           <t>Jeff Lima:</t>
         </r>
@@ -136,22 +416,22 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Segoe UI"/>
-            <family val="2"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
-Disciplina responsável ou à qual o requisito se aplica. Ex.: Arquitetura, Estrutura.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="E5" authorId="0" shapeId="0" xr:uid="{97AC1022-B243-44AF-9948-DB084DD23BAB}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
+Nome da propriedade dentro do Pset candidato.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Y5" authorId="0" shapeId="0" xr:uid="{BA2F3B25-B3D7-42C3-9C13-0A72F5E98317}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <charset val="1"/>
           </rPr>
           <t>Jeff Lima:</t>
         </r>
@@ -160,22 +440,22 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Segoe UI"/>
-            <family val="2"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
-Categoria autoral do Revit à qual o requisito se aplica. Ex.: Doors, Walls, Floors.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F5" authorId="0" shapeId="0" xr:uid="{EFBDE662-BA32-4D23-9E07-1EDE2120131C}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
+Regra objetiva que define aprovação ou reprovação do requisito.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Z5" authorId="0" shapeId="0" xr:uid="{9F9A4592-306B-482F-8E45-12749E42672C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <charset val="1"/>
           </rPr>
           <t>Jeff Lima:</t>
         </r>
@@ -184,22 +464,22 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Segoe UI"/>
-            <family val="2"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
-Família ou tipo usado como referência para avaliar o requisito. Não torna o requisito exclusivo desse exemplo.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G5" authorId="0" shapeId="0" xr:uid="{3818407D-0709-48D5-8E87-978AC8A34826}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
+Documento, planilha ou decisão do cliente que originou o requisito.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AA5" authorId="0" shapeId="0" xr:uid="{43CC9AD4-5B45-473B-AC3D-1792B0CE6D1E}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <charset val="1"/>
           </rPr>
           <t>Jeff Lima:</t>
         </r>
@@ -208,322 +488,10 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Segoe UI"/>
-            <family val="2"/>
+            <charset val="1"/>
           </rPr>
           <t xml:space="preserve">
-Indica onde o dado vive no Revit: instance, type ou unspecified.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H5" authorId="0" shapeId="0" xr:uid="{645D1314-194C-4089-AE8E-A1DAF527D04E}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t>Jeff Lima:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Unidade da grandeza. Ex.: mm, m², m³. Use N/A para textos, booleanos ou identificadores.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I5" authorId="0" shapeId="0" xr:uid="{A796D50C-A9AE-4B85-A719-7EB2232A961F}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t>Jeff Lima:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Natureza esperada do valor: text, integer, real, boolean, length, area, volume, identifier, date etc.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J5" authorId="0" shapeId="0" xr:uid="{2AD19DC1-789F-4EAF-A820-955E7A9320FA}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t>Jeff Lima:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Quantidade mínima e máxima de valores admitidos. 0..1 = opcional e único; 1 = obrigatório e único; 0..n = opcional e repetível; 1..n = pelo menos um. Orienta a cardinalidade do IDS.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K5" authorId="0" shapeId="0" xr:uid="{B60CC5C2-1BB2-45B1-A72D-5D9164297221}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t>Jeff Lima:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Lista, faixa, padrão ou enumeração admitida. Ex.: 30; 60; 90 ou Sim/Não. Deixe vazio quando livre.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="L5" authorId="0" shapeId="0" xr:uid="{ACB1B6F7-4A34-4EDD-BD52-28B14C72AC5C}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t>Jeff Lima:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Fase em que o dado se torna obrigatório. Ex.: Projeto executivo, Construção ou Operação.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M5" authorId="0" shapeId="0" xr:uid="{2289FD41-CA09-40CB-8DB8-D80FEC760B62}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t>Jeff Lima:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Versão exata do schema de entrega: IFC2X3, IFC4 ou IFC4.3. Não misture templates entre schemas.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="N5" authorId="0" shapeId="0" xr:uid="{7F990084-1255-4129-BE99-D7AFCFF80F04}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t>Jeff Lima:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Classe IFC inicialmente considerada para o objeto. É candidata até a validação técnica.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O5" authorId="0" shapeId="0" xr:uid="{9A8B6886-EDED-49C9-ACA5-19232D0806BE}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t>Jeff Lima:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-PredefinedType inicialmente considerado. Preencher somente quando existir e for aplicável no schema.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P5" authorId="0" shapeId="0" xr:uid="{61906A94-9BEE-4480-91E0-9E55600A648C}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t>Jeff Lima:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Pset inicialmente considerado. É apenas candidato; não combine automaticamente Pset e Qto.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Q5" authorId="0" shapeId="0" xr:uid="{755A232A-D378-4ECA-BC70-377FC2689830}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t>Jeff Lima:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Nome da propriedade IFC inicialmente considerada dentro do Pset candidato.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R5" authorId="0" shapeId="0" xr:uid="{B0679FEB-6BAC-40A2-870F-A76F2D73B04E}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t>Jeff Lima:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Regra objetiva de aprovação. Deve permitir que outra pessoa chegue à mesma decisão.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="S5" authorId="0" shapeId="0" xr:uid="{14E95F32-2DEF-4430-9FE4-2ED2AD84D25E}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t>Jeff Lima:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Documento, planilha, aba, linha ou identificador do requisito recebido do cliente.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="T5" authorId="0" shapeId="0" xr:uid="{764863F8-C16C-4CD8-8287-6AC55E1DBBF7}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t>Jeff Lima:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Segoe UI"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Contexto adicional, dúvidas, exceções ou premissas. Não usar para esconder requisito indefinido.</t>
+Hipóteses, pendências e decisões necessárias antes da geração do IDS.</t>
         </r>
       </text>
     </comment>
@@ -1502,7 +1470,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="248">
   <si>
     <t>TEMPLATE DE ENTRADA — REQUISITOS DE INFORMAÇÃO</t>
   </si>
@@ -1690,9 +1658,6 @@
     <t>Valor obrigatório para guarda-corpos no escopo</t>
   </si>
   <si>
-    <t>EXEMPLO — provável requisito customizado</t>
-  </si>
-  <si>
     <t>TEMPLATE DE SAÍDA — DECISÃO NATIVO × CUSTOMIZADO</t>
   </si>
   <si>
@@ -2179,12 +2144,6 @@
     <t>CALCULATED_ONLY</t>
   </si>
   <si>
-    <t>A skill consulta Revit, mapeamentos autorizados, schema IFC exato e evidências do export.</t>
-  </si>
-  <si>
-    <t>A skill separa origem autoral de ATTRIBUTE, Qto, Pset, associação, cálculo ou não verificado.</t>
-  </si>
-  <si>
     <t>Qto × Pset</t>
   </si>
   <si>
@@ -2195,13 +2154,73 @@
   </si>
   <si>
     <t>Aba produzida pela skill. Origem Revit e destino IFC são decisões separadas; CUSTOM_QTO exige prova no IFC exportado. Estados não verificáveis não liberam o gate.</t>
+  </si>
+  <si>
+    <t>Nome_Campo_Cliente</t>
+  </si>
+  <si>
+    <t>Parametro_Revit_Candidato</t>
+  </si>
+  <si>
+    <t>Origem_Revit_Tipo</t>
+  </si>
+  <si>
+    <t>Destino_IFC_Tipo_Candidato</t>
+  </si>
+  <si>
+    <t>Atributo_IFC_Candidato</t>
+  </si>
+  <si>
+    <t>QuantitySet_Candidato</t>
+  </si>
+  <si>
+    <t>QuantityName_Candidato</t>
+  </si>
+  <si>
+    <t>ResistenciaFogo</t>
+  </si>
+  <si>
+    <t>NATIVO</t>
+  </si>
+  <si>
+    <t>AreaPiso</t>
+  </si>
+  <si>
+    <t>TipoFixacaoGuardaCorpo</t>
+  </si>
+  <si>
+    <t>Tipo de Fixação</t>
+  </si>
+  <si>
+    <t>COMPARTILHADO</t>
+  </si>
+  <si>
+    <t>Pset_ClienteGuardaCorpo</t>
+  </si>
+  <si>
+    <t>EXEMPLO — provável requisito customizado; validar nome e governança do Pset</t>
+  </si>
+  <si>
+    <t>PROJETO</t>
+  </si>
+  <si>
+    <t>INEXISTENTE</t>
+  </si>
+  <si>
+    <t>EXTERNO</t>
+  </si>
+  <si>
+    <t>Regra: Codigo_Requisito é o identificador estável; Nome_Campo_Cliente, candidato Revit e destino IFC são conceitos distintos.</t>
+  </si>
+  <si>
+    <t>Destino IFC: use ATTRIBUTE, STANDARD_QTO/CUSTOM_QTO ou STANDARD_PSET/CUSTOM_PSET e preencha somente os campos correspondentes.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2258,6 +2277,19 @@
       <color indexed="81"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Segoe UI"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Segoe UI"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -2331,7 +2363,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2339,11 +2371,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -2356,11 +2384,580 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="66">
+  <dxfs count="73">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF2E74B5"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF14263A"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -3131,409 +3728,6 @@
           <color rgb="FFD5DEE6"/>
         </bottom>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FFFFFFFF"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FF2E74B5"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF14263A"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
     </dxf>
     <dxf>
       <border outline="0">
@@ -3560,78 +3754,85 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{70012B43-8741-4747-AB51-558D362B39EF}" name="tblEntradaRequisitos" displayName="tblEntradaRequisitos" ref="A5:T8" totalsRowShown="0" headerRowDxfId="43" dataDxfId="44" tableBorderDxfId="65">
-  <autoFilter ref="A5:T8" xr:uid="{70012B43-8741-4747-AB51-558D362B39EF}"/>
-  <tableColumns count="20">
-    <tableColumn id="1" xr3:uid="{BCFD0240-F9E1-43C6-BF2C-032C189B80CD}" name="Codigo_Requisito" dataDxfId="64"/>
-    <tableColumn id="2" xr3:uid="{BAEB5207-9C92-4762-BFDE-65D837EB5EA6}" name="Descricao" dataDxfId="63"/>
-    <tableColumn id="3" xr3:uid="{ADC800E5-5CCD-40C2-84C4-F96199E85D9C}" name="Finalidade_Uso" dataDxfId="62"/>
-    <tableColumn id="4" xr3:uid="{6942A4E1-12E8-4DF5-AE93-A6A1106BE0EF}" name="Disciplina" dataDxfId="61"/>
-    <tableColumn id="5" xr3:uid="{20241BDC-1AE9-4E9D-9438-9C5406DE9199}" name="Categoria_Revit" dataDxfId="60"/>
-    <tableColumn id="6" xr3:uid="{375471C2-8E7B-4BA5-A8C6-DE11D1695F98}" name="Familia_Tipo_Referencia" dataDxfId="59"/>
-    <tableColumn id="7" xr3:uid="{7664CF16-6EC4-411B-80D1-4CBBBDC6E490}" name="Escopo_Revit" dataDxfId="58"/>
-    <tableColumn id="8" xr3:uid="{12BD3E51-B93E-4783-BD2E-55ADF3275E81}" name="Unidade" dataDxfId="57"/>
-    <tableColumn id="9" xr3:uid="{E853E108-6839-4B92-AC1A-EB7ED17B2945}" name="Tipo_Dado_Esperado" dataDxfId="56"/>
-    <tableColumn id="10" xr3:uid="{F84BC120-7D95-4152-9C67-5D06D3ABDB54}" name="Cardinalidade" dataDxfId="55"/>
-    <tableColumn id="11" xr3:uid="{767651A9-0BEC-4E73-8C46-4B521E78AEE1}" name="Valores_Permitidos" dataDxfId="54"/>
-    <tableColumn id="12" xr3:uid="{4F84CC5F-6181-4389-ABE7-9A76F8AF910B}" name="Fase_Obrigatoriedade" dataDxfId="53"/>
-    <tableColumn id="13" xr3:uid="{4E68EA7D-16C2-4FA1-A492-E9E233F23174}" name="Schema_IFC" dataDxfId="52"/>
-    <tableColumn id="14" xr3:uid="{507F0EED-452D-4115-9EC6-23F1B426FAB9}" name="Classe_IFC_Candidata" dataDxfId="51"/>
-    <tableColumn id="15" xr3:uid="{9FADACD3-C7E2-4A68-A543-1D0582D1E834}" name="PredefinedType_Candidato" dataDxfId="50"/>
-    <tableColumn id="16" xr3:uid="{E2FE92AF-7F6D-4827-B8AD-C3BA8031BA96}" name="Pset_Candidato" dataDxfId="49"/>
-    <tableColumn id="17" xr3:uid="{8EBBCD26-104C-4BD0-ACA5-1548726E54DF}" name="Propriedade_Candidata" dataDxfId="48"/>
-    <tableColumn id="18" xr3:uid="{B42371CD-863B-49D3-8242-11ACB715B2C5}" name="Criterio_Aceitacao" dataDxfId="47"/>
-    <tableColumn id="19" xr3:uid="{6A832E3A-AAB8-48AF-A0AD-8974F38F55F0}" name="Fonte_Cliente" dataDxfId="46"/>
-    <tableColumn id="20" xr3:uid="{5A837F51-6C8C-4BE1-AA86-A660731F094F}" name="Observacoes" dataDxfId="45"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{70012B43-8741-4747-AB51-558D362B39EF}" name="tblEntradaRequisitos" displayName="tblEntradaRequisitos" ref="A5:AA8" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0" tableBorderDxfId="72">
+  <autoFilter ref="A5:AA8" xr:uid="{70012B43-8741-4747-AB51-558D362B39EF}"/>
+  <tableColumns count="27">
+    <tableColumn id="1" xr3:uid="{BCFD0240-F9E1-43C6-BF2C-032C189B80CD}" name="Codigo_Requisito" dataDxfId="28"/>
+    <tableColumn id="2" xr3:uid="{BAEB5207-9C92-4762-BFDE-65D837EB5EA6}" name="Nome_Campo_Cliente" dataDxfId="27"/>
+    <tableColumn id="3" xr3:uid="{ADC800E5-5CCD-40C2-84C4-F96199E85D9C}" name="Descricao" dataDxfId="26"/>
+    <tableColumn id="4" xr3:uid="{6942A4E1-12E8-4DF5-AE93-A6A1106BE0EF}" name="Finalidade_Uso" dataDxfId="25"/>
+    <tableColumn id="5" xr3:uid="{20241BDC-1AE9-4E9D-9438-9C5406DE9199}" name="Disciplina" dataDxfId="24"/>
+    <tableColumn id="6" xr3:uid="{375471C2-8E7B-4BA5-A8C6-DE11D1695F98}" name="Categoria_Revit" dataDxfId="23"/>
+    <tableColumn id="7" xr3:uid="{7664CF16-6EC4-411B-80D1-4CBBBDC6E490}" name="Familia_Tipo_Referencia" dataDxfId="22"/>
+    <tableColumn id="8" xr3:uid="{12BD3E51-B93E-4783-BD2E-55ADF3275E81}" name="Parametro_Revit_Candidato" dataDxfId="21"/>
+    <tableColumn id="9" xr3:uid="{E853E108-6839-4B92-AC1A-EB7ED17B2945}" name="Origem_Revit_Tipo" dataDxfId="20"/>
+    <tableColumn id="10" xr3:uid="{F84BC120-7D95-4152-9C67-5D06D3ABDB54}" name="Escopo_Revit" dataDxfId="19"/>
+    <tableColumn id="11" xr3:uid="{767651A9-0BEC-4E73-8C46-4B521E78AEE1}" name="Unidade" dataDxfId="18"/>
+    <tableColumn id="12" xr3:uid="{4F84CC5F-6181-4389-ABE7-9A76F8AF910B}" name="Tipo_Dado_Esperado" dataDxfId="17"/>
+    <tableColumn id="13" xr3:uid="{4E68EA7D-16C2-4FA1-A492-E9E233F23174}" name="Cardinalidade" dataDxfId="16"/>
+    <tableColumn id="14" xr3:uid="{507F0EED-452D-4115-9EC6-23F1B426FAB9}" name="Valores_Permitidos" dataDxfId="15"/>
+    <tableColumn id="15" xr3:uid="{9FADACD3-C7E2-4A68-A543-1D0582D1E834}" name="Fase_Obrigatoriedade" dataDxfId="14"/>
+    <tableColumn id="16" xr3:uid="{E2FE92AF-7F6D-4827-B8AD-C3BA8031BA96}" name="Schema_IFC" dataDxfId="13"/>
+    <tableColumn id="17" xr3:uid="{8EBBCD26-104C-4BD0-ACA5-1548726E54DF}" name="Classe_IFC_Candidata" dataDxfId="12"/>
+    <tableColumn id="18" xr3:uid="{B42371CD-863B-49D3-8242-11ACB715B2C5}" name="PredefinedType_Candidato" dataDxfId="11"/>
+    <tableColumn id="19" xr3:uid="{6A832E3A-AAB8-48AF-A0AD-8974F38F55F0}" name="Destino_IFC_Tipo_Candidato" dataDxfId="10"/>
+    <tableColumn id="20" xr3:uid="{5A837F51-6C8C-4BE1-AA86-A660731F094F}" name="Atributo_IFC_Candidato" dataDxfId="9"/>
+    <tableColumn id="21" xr3:uid="{79C09900-9C37-48C2-98E4-7EA53C8A8B5B}" name="QuantitySet_Candidato" dataDxfId="8"/>
+    <tableColumn id="22" xr3:uid="{4F8449F5-1F61-4D38-BA8E-DC1CC42C5688}" name="QuantityName_Candidato" dataDxfId="7"/>
+    <tableColumn id="23" xr3:uid="{6ABFFAB0-7B37-4E8A-8191-C00738DD6F9F}" name="Pset_Candidato" dataDxfId="6"/>
+    <tableColumn id="24" xr3:uid="{5B61C569-F850-43BC-8B36-FF40590D1BB7}" name="Propriedade_Candidata" dataDxfId="5"/>
+    <tableColumn id="25" xr3:uid="{70C98A92-51E9-409A-A4ED-703CCD11FDDF}" name="Criterio_Aceitacao" dataDxfId="4"/>
+    <tableColumn id="26" xr3:uid="{832C6844-614C-450E-89AC-53E38AEE53EA}" name="Fonte_Cliente" dataDxfId="3"/>
+    <tableColumn id="27" xr3:uid="{735381A9-D298-4118-8B05-FD35EFBDA9ED}" name="Observacoes" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1A55B9AA-85BD-489C-932C-E207E43AEB27}" name="tblSaidaMapeamento" displayName="tblSaidaMapeamento" ref="A5:AN8" totalsRowShown="0" headerRowDxfId="9" dataDxfId="10" tableBorderDxfId="42">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1A55B9AA-85BD-489C-932C-E207E43AEB27}" name="tblSaidaMapeamento" displayName="tblSaidaMapeamento" ref="A5:AN8" totalsRowShown="0" headerRowDxfId="38" dataDxfId="39" tableBorderDxfId="71">
   <autoFilter ref="A5:AN8" xr:uid="{1A55B9AA-85BD-489C-932C-E207E43AEB27}"/>
   <tableColumns count="40">
-    <tableColumn id="1" xr3:uid="{E981028E-4CCD-44EA-BDC9-C34246C28D21}" name="Codigo_Requisito" dataDxfId="41"/>
-    <tableColumn id="2" xr3:uid="{F9B8454A-A1B3-4BE1-8AB5-B55B83B50675}" name="Descricao_Normalizada" dataDxfId="40"/>
-    <tableColumn id="3" xr3:uid="{B2457B2C-15A5-4643-8097-F5F3ACAEA01F}" name="Classificacao" dataDxfId="39"/>
-    <tableColumn id="4" xr3:uid="{4D93E1F7-3119-4BAB-A90F-333A4D275046}" name="Acao" dataDxfId="38"/>
-    <tableColumn id="5" xr3:uid="{14706701-7382-4947-9560-5F3C95BA8C4B}" name="Justificativa_Decisao" dataDxfId="37"/>
-    <tableColumn id="6" xr3:uid="{0E660777-0E8C-4E54-B8DF-4A96516E8C90}" name="Nome_Parametro_Revit" dataDxfId="36"/>
-    <tableColumn id="7" xr3:uid="{9FC6D7E4-25B9-4AE0-88B5-E8B853328977}" name="Escopo_Revit" dataDxfId="35"/>
-    <tableColumn id="8" xr3:uid="{B2E411F2-5169-48AC-96AE-CB559C603D20}" name="Datatype_Revit" dataDxfId="34"/>
-    <tableColumn id="9" xr3:uid="{7DAFEEDB-EF68-405B-B8E4-48AD2E2E7B40}" name="Categorias_Revit" dataDxfId="33"/>
-    <tableColumn id="10" xr3:uid="{F1F07C04-E357-4B64-B5F5-A0B10D697210}" name="GUID" dataDxfId="32"/>
-    <tableColumn id="11" xr3:uid="{4573903C-C7D9-451C-B8F5-5C58A2675EFE}" name="Grupo_Parametro" dataDxfId="31"/>
-    <tableColumn id="12" xr3:uid="{68CE38D8-DCFD-4078-9B1E-AA80F2926F66}" name="Schema_IFC" dataDxfId="30"/>
-    <tableColumn id="13" xr3:uid="{090B31C4-2BB9-4AAB-BB75-01453F756802}" name="Classe_IFC" dataDxfId="29"/>
-    <tableColumn id="14" xr3:uid="{B2837CBD-E0E7-48E4-8EB0-D133F5B659DC}" name="PredefinedType" dataDxfId="28"/>
-    <tableColumn id="15" xr3:uid="{1A2186AC-A3CE-4A17-B367-A316C241BBF8}" name="Destino_IFC_Tipo" dataDxfId="27"/>
-    <tableColumn id="32" xr3:uid="{4162F999-A46E-470E-A138-654D3FEF72E1}" name="Atributo_IFC" dataDxfId="8"/>
-    <tableColumn id="33" xr3:uid="{D5E523EC-AADA-44CF-A55D-177F021032ED}" name="QuantitySet" dataDxfId="7"/>
-    <tableColumn id="34" xr3:uid="{24AE3DFB-32CC-41C6-BCAE-E7732DA4E539}" name="QuantityName" dataDxfId="6"/>
-    <tableColumn id="35" xr3:uid="{3BBCA9E3-AF73-4A00-B6B3-39EFBC16F73C}" name="QuantityType" dataDxfId="5"/>
-    <tableColumn id="36" xr3:uid="{55F3BDE0-8704-4575-A8D0-EB34447518DA}" name="MethodOfMeasurement" dataDxfId="4"/>
-    <tableColumn id="37" xr3:uid="{3F749E5E-2446-4A0E-AF27-AD5EF11A7E22}" name="Formula_Calculo" dataDxfId="3"/>
-    <tableColumn id="38" xr3:uid="{3D268C46-D848-4F3B-A1B4-424FBAE64C12}" name="Pset" dataDxfId="2"/>
-    <tableColumn id="39" xr3:uid="{6F81026C-B4F5-4B5E-A265-6FB0BDD3C6BB}" name="Propriedade_IFC" dataDxfId="1"/>
-    <tableColumn id="40" xr3:uid="{C9C66B86-4A1E-49CD-AF8B-C1B034BE74B4}" name="Datatype_IFC" dataDxfId="0"/>
-    <tableColumn id="16" xr3:uid="{03622A26-7283-4252-AD58-5D0844BA7D81}" name="Associacao_Material" dataDxfId="26"/>
-    <tableColumn id="17" xr3:uid="{0BE30617-6140-4B20-938F-345BE1A5B83F}" name="Metodo_Mapeamento" dataDxfId="25"/>
-    <tableColumn id="18" xr3:uid="{CA9DF3D9-1F5F-47ED-AE26-B67F89E03A2B}" name="Origem_Dado" dataDxfId="24"/>
-    <tableColumn id="19" xr3:uid="{071D62D5-1B6C-4D61-856A-F5922CC8BB46}" name="Source_Kind" dataDxfId="23"/>
-    <tableColumn id="20" xr3:uid="{C8313205-5CCA-4FD9-AEA7-EA27A433F1EB}" name="Arquivo_Fonte" dataDxfId="22"/>
-    <tableColumn id="21" xr3:uid="{DDE490D1-8952-47EB-991E-9CB2D4A8EACA}" name="Linha_Fonte" dataDxfId="21"/>
-    <tableColumn id="22" xr3:uid="{BDD71F5D-B366-4375-9B64-E679009C90B8}" name="Entidade_Exportada_Comprovada" dataDxfId="20"/>
-    <tableColumn id="23" xr3:uid="{28A7CC09-C4AD-4410-BEBB-555F89561CC4}" name="Evidencia_Inspecao_IFC" dataDxfId="19"/>
-    <tableColumn id="24" xr3:uid="{1C2C51EB-5A6A-4388-A671-76B2CED71234}" name="Conflito_Detectado" dataDxfId="18"/>
-    <tableColumn id="25" xr3:uid="{DC8F0597-56FA-4518-8040-2753081FC2E9}" name="Limitacoes" dataDxfId="17"/>
-    <tableColumn id="26" xr3:uid="{31FEC073-A8D1-45E5-BA27-A207E6C60117}" name="Requer_Aprovacao_Humana" dataDxfId="16"/>
-    <tableColumn id="27" xr3:uid="{A035FABF-7925-4F28-B1E5-4425594E2F29}" name="Responsavel_Aprovacao" dataDxfId="15"/>
-    <tableColumn id="28" xr3:uid="{5C6F6B56-A97B-466F-AE96-9F6BB90C3C4D}" name="Status_Decisao" dataDxfId="14"/>
-    <tableColumn id="29" xr3:uid="{1F4FEC58-FD7F-4203-B6BC-A6E05303E3F3}" name="Versao_Mapeamento" dataDxfId="13"/>
-    <tableColumn id="30" xr3:uid="{F5960338-8224-4877-8DD8-B2D39A7E6241}" name="Data_Analise" dataDxfId="12"/>
-    <tableColumn id="31" xr3:uid="{A7950B61-C6EC-4C84-AAB1-AB524293B49C}" name="Observacoes" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{E981028E-4CCD-44EA-BDC9-C34246C28D21}" name="Codigo_Requisito" dataDxfId="70"/>
+    <tableColumn id="2" xr3:uid="{F9B8454A-A1B3-4BE1-8AB5-B55B83B50675}" name="Descricao_Normalizada" dataDxfId="69"/>
+    <tableColumn id="3" xr3:uid="{B2457B2C-15A5-4643-8097-F5F3ACAEA01F}" name="Classificacao" dataDxfId="68"/>
+    <tableColumn id="4" xr3:uid="{4D93E1F7-3119-4BAB-A90F-333A4D275046}" name="Acao" dataDxfId="67"/>
+    <tableColumn id="5" xr3:uid="{14706701-7382-4947-9560-5F3C95BA8C4B}" name="Justificativa_Decisao" dataDxfId="66"/>
+    <tableColumn id="6" xr3:uid="{0E660777-0E8C-4E54-B8DF-4A96516E8C90}" name="Nome_Parametro_Revit" dataDxfId="65"/>
+    <tableColumn id="7" xr3:uid="{9FC6D7E4-25B9-4AE0-88B5-E8B853328977}" name="Escopo_Revit" dataDxfId="64"/>
+    <tableColumn id="8" xr3:uid="{B2E411F2-5169-48AC-96AE-CB559C603D20}" name="Datatype_Revit" dataDxfId="63"/>
+    <tableColumn id="9" xr3:uid="{7DAFEEDB-EF68-405B-B8E4-48AD2E2E7B40}" name="Categorias_Revit" dataDxfId="62"/>
+    <tableColumn id="10" xr3:uid="{F1F07C04-E357-4B64-B5F5-A0B10D697210}" name="GUID" dataDxfId="61"/>
+    <tableColumn id="11" xr3:uid="{4573903C-C7D9-451C-B8F5-5C58A2675EFE}" name="Grupo_Parametro" dataDxfId="60"/>
+    <tableColumn id="12" xr3:uid="{68CE38D8-DCFD-4078-9B1E-AA80F2926F66}" name="Schema_IFC" dataDxfId="59"/>
+    <tableColumn id="13" xr3:uid="{090B31C4-2BB9-4AAB-BB75-01453F756802}" name="Classe_IFC" dataDxfId="58"/>
+    <tableColumn id="14" xr3:uid="{B2837CBD-E0E7-48E4-8EB0-D133F5B659DC}" name="PredefinedType" dataDxfId="57"/>
+    <tableColumn id="15" xr3:uid="{1A2186AC-A3CE-4A17-B367-A316C241BBF8}" name="Destino_IFC_Tipo" dataDxfId="56"/>
+    <tableColumn id="32" xr3:uid="{4162F999-A46E-470E-A138-654D3FEF72E1}" name="Atributo_IFC" dataDxfId="37"/>
+    <tableColumn id="33" xr3:uid="{D5E523EC-AADA-44CF-A55D-177F021032ED}" name="QuantitySet" dataDxfId="36"/>
+    <tableColumn id="34" xr3:uid="{24AE3DFB-32CC-41C6-BCAE-E7732DA4E539}" name="QuantityName" dataDxfId="35"/>
+    <tableColumn id="35" xr3:uid="{3BBCA9E3-AF73-4A00-B6B3-39EFBC16F73C}" name="QuantityType" dataDxfId="34"/>
+    <tableColumn id="36" xr3:uid="{55F3BDE0-8704-4575-A8D0-EB34447518DA}" name="MethodOfMeasurement" dataDxfId="33"/>
+    <tableColumn id="37" xr3:uid="{3F749E5E-2446-4A0E-AF27-AD5EF11A7E22}" name="Formula_Calculo" dataDxfId="32"/>
+    <tableColumn id="38" xr3:uid="{3D268C46-D848-4F3B-A1B4-424FBAE64C12}" name="Pset" dataDxfId="31"/>
+    <tableColumn id="39" xr3:uid="{6F81026C-B4F5-4B5E-A265-6FB0BDD3C6BB}" name="Propriedade_IFC" dataDxfId="30"/>
+    <tableColumn id="40" xr3:uid="{C9C66B86-4A1E-49CD-AF8B-C1B034BE74B4}" name="Datatype_IFC" dataDxfId="29"/>
+    <tableColumn id="16" xr3:uid="{03622A26-7283-4252-AD58-5D0844BA7D81}" name="Associacao_Material" dataDxfId="55"/>
+    <tableColumn id="17" xr3:uid="{0BE30617-6140-4B20-938F-345BE1A5B83F}" name="Metodo_Mapeamento" dataDxfId="54"/>
+    <tableColumn id="18" xr3:uid="{CA9DF3D9-1F5F-47ED-AE26-B67F89E03A2B}" name="Origem_Dado" dataDxfId="53"/>
+    <tableColumn id="19" xr3:uid="{071D62D5-1B6C-4D61-856A-F5922CC8BB46}" name="Source_Kind" dataDxfId="52"/>
+    <tableColumn id="20" xr3:uid="{C8313205-5CCA-4FD9-AEA7-EA27A433F1EB}" name="Arquivo_Fonte" dataDxfId="51"/>
+    <tableColumn id="21" xr3:uid="{DDE490D1-8952-47EB-991E-9CB2D4A8EACA}" name="Linha_Fonte" dataDxfId="50"/>
+    <tableColumn id="22" xr3:uid="{BDD71F5D-B366-4375-9B64-E679009C90B8}" name="Entidade_Exportada_Comprovada" dataDxfId="49"/>
+    <tableColumn id="23" xr3:uid="{28A7CC09-C4AD-4410-BEBB-555F89561CC4}" name="Evidencia_Inspecao_IFC" dataDxfId="48"/>
+    <tableColumn id="24" xr3:uid="{1C2C51EB-5A6A-4388-A671-76B2CED71234}" name="Conflito_Detectado" dataDxfId="47"/>
+    <tableColumn id="25" xr3:uid="{DC8F0597-56FA-4518-8040-2753081FC2E9}" name="Limitacoes" dataDxfId="46"/>
+    <tableColumn id="26" xr3:uid="{31FEC073-A8D1-45E5-BA27-A207E6C60117}" name="Requer_Aprovacao_Humana" dataDxfId="45"/>
+    <tableColumn id="27" xr3:uid="{A035FABF-7925-4F28-B1E5-4425594E2F29}" name="Responsavel_Aprovacao" dataDxfId="44"/>
+    <tableColumn id="28" xr3:uid="{5C6F6B56-A97B-466F-AE96-9F6BB90C3C4D}" name="Status_Decisao" dataDxfId="43"/>
+    <tableColumn id="29" xr3:uid="{1F4FEC58-FD7F-4203-B6BC-A6E05303E3F3}" name="Versao_Mapeamento" dataDxfId="42"/>
+    <tableColumn id="30" xr3:uid="{F5960338-8224-4877-8DD8-B2D39A7E6241}" name="Data_Analise" dataDxfId="41"/>
+    <tableColumn id="31" xr3:uid="{A7950B61-C6EC-4C84-AAB1-AB524293B49C}" name="Observacoes" dataDxfId="40"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3976,32 +4177,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54296401-7BB5-4C16-95CB-A0A7BED3DEA2}">
-  <dimension ref="A1:T8"/>
+  <dimension ref="A1:AA8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="62" customWidth="1"/>
-    <col min="3" max="3" width="31.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="27.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="25.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="26" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="30.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="27" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="44.85546875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="64.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="73.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="31.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="25.42578125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="26" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="32" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="23.85546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="27" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="44.85546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="73" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:27" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -4025,8 +4233,8 @@
       <c r="S1" s="2"/>
       <c r="T1" s="2"/>
     </row>
-    <row r="2" spans="1:20" ht="45" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
+    <row r="2" spans="1:27" ht="45" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="3"/>
@@ -4049,7 +4257,7 @@
       <c r="S2" s="3"/>
       <c r="T2" s="3"/>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -4071,240 +4279,308 @@
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
     </row>
-    <row r="5" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="7" t="s">
+    <row r="5" spans="1:27" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="C5" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="D5" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="E5" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="F5" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="G5" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="H5" s="12" t="s">
+        <v>229</v>
+      </c>
+      <c r="I5" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="J5" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="K5" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="7" t="s">
+      <c r="L5" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="J5" s="7" t="s">
+      <c r="M5" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="K5" s="7" t="s">
+      <c r="N5" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="L5" s="7" t="s">
+      <c r="O5" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="M5" s="7" t="s">
+      <c r="P5" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="N5" s="7" t="s">
+      <c r="Q5" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="O5" s="7" t="s">
+      <c r="R5" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="P5" s="7" t="s">
+      <c r="S5" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="T5" s="12" t="s">
+        <v>232</v>
+      </c>
+      <c r="U5" s="12" t="s">
+        <v>233</v>
+      </c>
+      <c r="V5" s="12" t="s">
+        <v>234</v>
+      </c>
+      <c r="W5" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="Q5" s="7" t="s">
+      <c r="X5" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="R5" s="7" t="s">
+      <c r="Y5" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="S5" s="7" t="s">
+      <c r="Z5" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="T5" s="7" t="s">
+      <c r="AA5" s="12" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="13" t="s">
+        <v>235</v>
+      </c>
+      <c r="C6" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="D6" s="13" t="s">
         <v>24</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="E6" s="13" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="F6" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="G6" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="H6" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="I6" s="13" t="s">
+        <v>236</v>
+      </c>
+      <c r="J6" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="K6" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="L6" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="J6" s="5">
+      <c r="M6" s="13">
         <v>1</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="N6" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="L6" s="5" t="s">
+      <c r="O6" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="M6" s="5" t="s">
+      <c r="P6" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="N6" s="5" t="s">
+      <c r="Q6" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="O6" s="5"/>
-      <c r="P6" s="5" t="s">
+      <c r="R6" s="13"/>
+      <c r="S6" s="13" t="s">
+        <v>206</v>
+      </c>
+      <c r="T6" s="13"/>
+      <c r="U6" s="13"/>
+      <c r="V6" s="13"/>
+      <c r="W6" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="Q6" s="5" t="s">
+      <c r="X6" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="R6" s="5" t="s">
+      <c r="Y6" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="S6" s="5" t="s">
+      <c r="Z6" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="T6" s="5" t="s">
+      <c r="AA6" s="13" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A7" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="14" t="s">
+        <v>237</v>
+      </c>
+      <c r="C7" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="D7" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="E7" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="F7" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="14"/>
+      <c r="H7" s="14" t="s">
+        <v>108</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="J7" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="H7" s="6" t="s">
+      <c r="K7" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="L7" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="J7" s="6">
+      <c r="M7" s="14">
         <v>1</v>
       </c>
-      <c r="K7" s="6"/>
-      <c r="L7" s="6" t="s">
+      <c r="N7" s="14"/>
+      <c r="O7" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="M7" s="6" t="s">
+      <c r="P7" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="N7" s="6" t="s">
+      <c r="Q7" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="O7" s="6" t="s">
+      <c r="R7" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="P7" s="6" t="s">
+      <c r="S7" s="14" t="s">
+        <v>220</v>
+      </c>
+      <c r="T7" s="14"/>
+      <c r="U7" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="Q7" s="6" t="s">
+      <c r="V7" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="R7" s="6" t="s">
+      <c r="W7" s="14"/>
+      <c r="X7" s="14"/>
+      <c r="Y7" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="S7" s="6" t="s">
+      <c r="Z7" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="T7" s="6" t="s">
+      <c r="AA7" s="14" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A8" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="14" t="s">
+        <v>238</v>
+      </c>
+      <c r="C8" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="D8" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="E8" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6" t="s">
+      <c r="G8" s="14"/>
+      <c r="H8" s="14" t="s">
+        <v>239</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>240</v>
+      </c>
+      <c r="J8" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="H8" s="6" t="s">
+      <c r="K8" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="I8" s="6" t="s">
+      <c r="L8" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="J8" s="6">
+      <c r="M8" s="14">
         <v>1</v>
       </c>
-      <c r="K8" s="6" t="s">
+      <c r="N8" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="L8" s="6" t="s">
+      <c r="O8" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="M8" s="6" t="s">
+      <c r="P8" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="N8" s="6" t="s">
+      <c r="Q8" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="O8" s="6"/>
-      <c r="P8" s="6"/>
-      <c r="Q8" s="6" t="s">
+      <c r="R8" s="14"/>
+      <c r="S8" s="14" t="s">
+        <v>217</v>
+      </c>
+      <c r="T8" s="14"/>
+      <c r="U8" s="14"/>
+      <c r="V8" s="14"/>
+      <c r="W8" s="14" t="s">
+        <v>241</v>
+      </c>
+      <c r="X8" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="R8" s="6" t="s">
+      <c r="Y8" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="S8" s="6" t="s">
+      <c r="Z8" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="T8" s="6" t="s">
-        <v>62</v>
+      <c r="AA8" s="14" t="s">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -4401,7 +4677,7 @@
   <sheetData>
     <row r="1" spans="1:40" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4444,8 +4720,8 @@
       <c r="AN1" s="1"/>
     </row>
     <row r="2" spans="1:40" ht="45" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
-        <v>230</v>
+      <c r="A2" s="10" t="s">
+        <v>227</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -4530,425 +4806,425 @@
       <c r="AN3" s="3"/>
     </row>
     <row r="5" spans="1:40" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="D5" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="E5" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="F5" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="G5" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="H5" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="G5" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="H5" s="11" t="s">
+      <c r="I5" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="I5" s="11" t="s">
+      <c r="J5" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="J5" s="11" t="s">
+      <c r="K5" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="K5" s="11" t="s">
+      <c r="L5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="M5" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="L5" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="M5" s="11" t="s">
+      <c r="N5" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="N5" s="11" t="s">
+      <c r="O5" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="P5" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="Q5" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="R5" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="S5" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="T5" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="U5" s="11" t="s">
+        <v>202</v>
+      </c>
+      <c r="V5" s="11" t="s">
+        <v>203</v>
+      </c>
+      <c r="W5" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="O5" s="13" t="s">
-        <v>197</v>
-      </c>
-      <c r="P5" s="13" t="s">
-        <v>198</v>
-      </c>
-      <c r="Q5" s="13" t="s">
-        <v>199</v>
-      </c>
-      <c r="R5" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="S5" s="13" t="s">
-        <v>201</v>
-      </c>
-      <c r="T5" s="13" t="s">
-        <v>202</v>
-      </c>
-      <c r="U5" s="13" t="s">
-        <v>203</v>
-      </c>
-      <c r="V5" s="13" t="s">
+      <c r="X5" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="Y5" s="11" t="s">
         <v>204</v>
       </c>
-      <c r="W5" s="13" t="s">
-        <v>75</v>
-      </c>
-      <c r="X5" s="13" t="s">
+      <c r="Z5" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="Y5" s="13" t="s">
+      <c r="AA5" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="AB5" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="AC5" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="AD5" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="AE5" s="11" t="s">
         <v>205</v>
       </c>
-      <c r="Z5" s="13" t="s">
-        <v>77</v>
-      </c>
-      <c r="AA5" s="13" t="s">
-        <v>78</v>
-      </c>
-      <c r="AB5" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="AC5" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="AD5" s="13" t="s">
+      <c r="AF5" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="AE5" s="13" t="s">
-        <v>206</v>
-      </c>
-      <c r="AF5" s="13" t="s">
+      <c r="AG5" s="11" t="s">
         <v>82</v>
       </c>
-      <c r="AG5" s="13" t="s">
+      <c r="AH5" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="AH5" s="13" t="s">
+      <c r="AI5" s="11" t="s">
         <v>84</v>
       </c>
-      <c r="AI5" s="13" t="s">
+      <c r="AJ5" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="AJ5" s="13" t="s">
+      <c r="AK5" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="AK5" s="13" t="s">
+      <c r="AL5" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="AL5" s="13" t="s">
+      <c r="AM5" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="AM5" s="13" t="s">
-        <v>89</v>
-      </c>
-      <c r="AN5" s="13" t="s">
+      <c r="AN5" s="11" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="E6" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="F6" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="G6" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="J6" s="7"/>
+      <c r="K6" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G6" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="I6" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9" t="s">
+      <c r="L6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="M6" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="N6" s="7"/>
+      <c r="O6" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="P6" s="5"/>
+      <c r="Q6" s="5"/>
+      <c r="R6" s="5"/>
+      <c r="S6" s="5"/>
+      <c r="T6" s="5"/>
+      <c r="U6" s="5"/>
+      <c r="V6" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="W6" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="X6" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="L6" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="M6" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="N6" s="9"/>
-      <c r="O6" s="6" t="s">
+      <c r="Y6" s="5"/>
+      <c r="Z6" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="AA6" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="AB6" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="AC6" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="AD6" s="5"/>
+      <c r="AE6" s="5" t="s">
         <v>207</v>
       </c>
-      <c r="P6" s="6"/>
-      <c r="Q6" s="6"/>
-      <c r="R6" s="6"/>
-      <c r="S6" s="6"/>
-      <c r="T6" s="6"/>
-      <c r="U6" s="6"/>
-      <c r="V6" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="W6" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="X6" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="Y6" s="6"/>
-      <c r="Z6" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="AA6" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="AB6" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="AC6" s="6" t="s">
+      <c r="AF6" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="AD6" s="6"/>
-      <c r="AE6" s="6" t="s">
+      <c r="AG6" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="AH6" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="AI6" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="AJ6" s="5"/>
+      <c r="AK6" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="AL6" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="AF6" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="AG6" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="AH6" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="AI6" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="AJ6" s="6"/>
-      <c r="AK6" s="6" t="s">
+      <c r="AM6" s="8">
+        <v>46228</v>
+      </c>
+      <c r="AN6" s="5" t="s">
         <v>104</v>
-      </c>
-      <c r="AL6" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="AM6" s="10">
-        <v>46228</v>
-      </c>
-      <c r="AN6" s="6" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="7" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="E7" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="F7" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="G7" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="G7" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="J7" s="6"/>
-      <c r="K7" s="6" t="s">
+      <c r="L7" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="N7" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="O7" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="P7" s="5"/>
+      <c r="Q7" s="5"/>
+      <c r="R7" s="5"/>
+      <c r="S7" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="T7" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="U7" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="V7" s="5"/>
+      <c r="W7" s="5"/>
+      <c r="X7" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="L7" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="M7" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="N7" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="O7" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="P7" s="6"/>
-      <c r="Q7" s="6"/>
-      <c r="R7" s="6"/>
-      <c r="S7" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="T7" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="U7" s="6" t="s">
+      <c r="Y7" s="5"/>
+      <c r="Z7" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="V7" s="6"/>
-      <c r="W7" s="6"/>
-      <c r="X7" s="6" t="s">
+      <c r="AA7" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="Y7" s="6"/>
-      <c r="Z7" s="6" t="s">
+      <c r="AB7" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="AC7" s="5"/>
+      <c r="AD7" s="5"/>
+      <c r="AE7" s="5"/>
+      <c r="AF7" s="5" t="s">
         <v>214</v>
       </c>
-      <c r="AA7" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="AB7" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="AC7" s="6"/>
-      <c r="AD7" s="6"/>
-      <c r="AE7" s="6"/>
-      <c r="AF7" s="6" t="s">
+      <c r="AG7" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="AH7" s="5" t="s">
         <v>215</v>
       </c>
-      <c r="AG7" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="AH7" s="6" t="s">
+      <c r="AI7" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="AJ7" s="5"/>
+      <c r="AK7" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="AL7" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="AM7" s="8">
+        <v>46228</v>
+      </c>
+      <c r="AN7" s="5" t="s">
         <v>216</v>
-      </c>
-      <c r="AI7" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="AJ7" s="6"/>
-      <c r="AK7" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="AL7" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="AM7" s="10">
-        <v>46228</v>
-      </c>
-      <c r="AN7" s="6" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="8" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="E8" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="J8" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="K8" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="N8" s="5"/>
+      <c r="O8" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="P8" s="5"/>
+      <c r="Q8" s="5"/>
+      <c r="R8" s="5"/>
+      <c r="S8" s="5"/>
+      <c r="T8" s="5"/>
+      <c r="U8" s="5"/>
+      <c r="V8" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="W8" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G8" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="K8" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="L8" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="M8" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="N8" s="6"/>
-      <c r="O8" s="6" t="s">
+      <c r="X8" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="Y8" s="5"/>
+      <c r="Z8" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="AA8" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="AB8" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="AC8" s="5"/>
+      <c r="AD8" s="5"/>
+      <c r="AE8" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="AF8" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="AG8" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="AH8" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="P8" s="6"/>
-      <c r="Q8" s="6"/>
-      <c r="R8" s="6"/>
-      <c r="S8" s="6"/>
-      <c r="T8" s="6"/>
-      <c r="U8" s="6"/>
-      <c r="V8" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="W8" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="X8" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="Y8" s="6"/>
-      <c r="Z8" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="AA8" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="AB8" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="AC8" s="6"/>
-      <c r="AD8" s="6"/>
-      <c r="AE8" s="6" t="s">
+      <c r="AI8" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="AJ8" s="5"/>
+      <c r="AK8" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="AL8" s="5" t="s">
         <v>208</v>
       </c>
-      <c r="AF8" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="AG8" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="AH8" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="AI8" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="AJ8" s="6"/>
-      <c r="AK8" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="AL8" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="AM8" s="10">
+      <c r="AM8" s="8">
         <v>46228</v>
       </c>
-      <c r="AN8" s="6" t="s">
-        <v>105</v>
+      <c r="AN8" s="5" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -5014,7 +5290,7 @@
   <sheetPr>
     <tabColor rgb="FF667587"/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.28515625" bestFit="1" customWidth="1"/>
@@ -5026,49 +5302,53 @@
     <col min="8" max="8" width="13.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="28.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="F1" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="D1" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="F1" s="8" t="s">
+      <c r="G1" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="H1" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="H1" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="I1" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>197</v>
+      <c r="K1" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="L1" t="s">
+        <v>230</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C2" t="s">
         <v>44</v>
@@ -5077,214 +5357,238 @@
         <v>33</v>
       </c>
       <c r="E2" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="F2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G2" t="s">
         <v>30</v>
       </c>
       <c r="H2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I2" t="s">
         <v>25</v>
       </c>
       <c r="J2" t="s">
+        <v>130</v>
+      </c>
+      <c r="K2" t="s">
+        <v>219</v>
+      </c>
+      <c r="L2" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>131</v>
       </c>
-      <c r="K2" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="B3" t="s">
         <v>132</v>
-      </c>
-      <c r="B3" t="s">
-        <v>133</v>
       </c>
       <c r="C3" t="s">
         <v>28</v>
       </c>
       <c r="D3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E3" t="s">
+        <v>103</v>
+      </c>
+      <c r="F3" t="s">
+        <v>100</v>
+      </c>
+      <c r="G3" t="s">
         <v>134</v>
-      </c>
-      <c r="E3" t="s">
-        <v>104</v>
-      </c>
-      <c r="F3" t="s">
-        <v>101</v>
-      </c>
-      <c r="G3" t="s">
-        <v>135</v>
       </c>
       <c r="H3">
         <v>1</v>
       </c>
       <c r="I3" t="s">
+        <v>135</v>
+      </c>
+      <c r="J3" t="s">
         <v>136</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
+        <v>220</v>
+      </c>
+      <c r="L3" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>137</v>
       </c>
-      <c r="K3" t="s">
+      <c r="B4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" t="s">
+        <v>138</v>
+      </c>
+      <c r="D4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E4" t="s">
+        <v>140</v>
+      </c>
+      <c r="G4" t="s">
+        <v>141</v>
+      </c>
+      <c r="H4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I4" t="s">
+        <v>143</v>
+      </c>
+      <c r="J4" t="s">
+        <v>144</v>
+      </c>
+      <c r="K4" t="s">
         <v>221</v>
       </c>
+      <c r="L4" t="s">
+        <v>243</v>
+      </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>138</v>
-      </c>
-      <c r="B4" t="s">
-        <v>91</v>
-      </c>
-      <c r="C4" t="s">
-        <v>139</v>
-      </c>
-      <c r="D4" t="s">
-        <v>140</v>
-      </c>
-      <c r="E4" t="s">
-        <v>141</v>
-      </c>
-      <c r="G4" t="s">
-        <v>142</v>
-      </c>
-      <c r="H4" t="s">
-        <v>143</v>
-      </c>
-      <c r="I4" t="s">
-        <v>144</v>
-      </c>
-      <c r="J4" t="s">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B5" t="s">
+        <v>106</v>
+      </c>
+      <c r="E5" t="s">
         <v>145</v>
       </c>
-      <c r="K4" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>114</v>
-      </c>
-      <c r="B5" t="s">
-        <v>107</v>
-      </c>
-      <c r="E5" t="s">
+      <c r="G5" t="s">
         <v>146</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>147</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>148</v>
-      </c>
-      <c r="I5" t="s">
-        <v>149</v>
       </c>
       <c r="J5" t="s">
         <v>32</v>
       </c>
       <c r="K5" t="s">
-        <v>207</v>
+        <v>206</v>
+      </c>
+      <c r="L5" t="s">
+        <v>105</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>149</v>
+      </c>
+      <c r="B6" t="s">
         <v>150</v>
       </c>
-      <c r="B6" t="s">
+      <c r="E6" t="s">
+        <v>123</v>
+      </c>
+      <c r="G6" t="s">
         <v>151</v>
       </c>
-      <c r="E6" t="s">
-        <v>124</v>
-      </c>
-      <c r="G6" t="s">
+      <c r="I6" t="s">
         <v>152</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>153</v>
       </c>
-      <c r="J6" t="s">
+      <c r="K6" t="s">
+        <v>217</v>
+      </c>
+      <c r="L6" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>105</v>
+      </c>
+      <c r="B7" t="s">
         <v>154</v>
-      </c>
-      <c r="K6" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>106</v>
-      </c>
-      <c r="B7" t="s">
-        <v>155</v>
       </c>
       <c r="G7" t="s">
         <v>46</v>
       </c>
       <c r="I7" t="s">
+        <v>155</v>
+      </c>
+      <c r="J7" t="s">
         <v>156</v>
       </c>
-      <c r="J7" t="s">
+      <c r="K7" t="s">
+        <v>222</v>
+      </c>
+      <c r="L7" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>157</v>
       </c>
-      <c r="K7" t="s">
+      <c r="B8" t="s">
+        <v>158</v>
+      </c>
+      <c r="G8" t="s">
+        <v>159</v>
+      </c>
+      <c r="I8" t="s">
+        <v>160</v>
+      </c>
+      <c r="K8" t="s">
         <v>223</v>
       </c>
+      <c r="L8" t="s">
+        <v>245</v>
+      </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>158</v>
-      </c>
-      <c r="B8" t="s">
-        <v>159</v>
-      </c>
-      <c r="G8" t="s">
-        <v>160</v>
-      </c>
-      <c r="I8" t="s">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>161</v>
       </c>
-      <c r="K8" t="s">
-        <v>224</v>
+      <c r="G9" t="s">
+        <v>162</v>
+      </c>
+      <c r="I9" t="s">
+        <v>163</v>
+      </c>
+      <c r="K9" t="s">
+        <v>209</v>
+      </c>
+      <c r="L9" t="s">
+        <v>209</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>162</v>
-      </c>
-      <c r="G9" t="s">
-        <v>163</v>
-      </c>
-      <c r="I9" t="s">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>164</v>
       </c>
-      <c r="K9" t="s">
-        <v>210</v>
+      <c r="G10" t="s">
+        <v>165</v>
+      </c>
+      <c r="I10" t="s">
+        <v>166</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>165</v>
-      </c>
-      <c r="G10" t="s">
-        <v>166</v>
-      </c>
-      <c r="I10" t="s">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>123</v>
+      </c>
+      <c r="G11" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>124</v>
-      </c>
-      <c r="G11" t="s">
+      <c r="I11" t="s">
         <v>168</v>
-      </c>
-      <c r="I11" t="s">
-        <v>169</v>
       </c>
     </row>
   </sheetData>
@@ -5300,15 +5604,15 @@
   <dimension ref="A1:H18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="90.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="70.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="46.7109375" customWidth="1"/>
+    <col min="2" max="2" width="81" customWidth="1"/>
     <col min="3" max="3" width="23.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="33.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -5320,7 +5624,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -5342,134 +5646,134 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>173</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>174</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="C6" t="s">
         <v>176</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>177</v>
       </c>
-      <c r="D6" t="s">
-        <v>178</v>
-      </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2</v>
       </c>
-      <c r="B7" t="s">
-        <v>225</v>
+      <c r="B7" s="15" t="s">
+        <v>246</v>
       </c>
       <c r="C7" t="s">
+        <v>178</v>
+      </c>
+      <c r="D7" t="s">
         <v>179</v>
       </c>
-      <c r="D7" t="s">
-        <v>180</v>
-      </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>3</v>
       </c>
-      <c r="B8" t="s">
-        <v>226</v>
+      <c r="B8" s="15" t="s">
+        <v>247</v>
       </c>
       <c r="C8" t="s">
+        <v>180</v>
+      </c>
+      <c r="D8" t="s">
         <v>181</v>
-      </c>
-      <c r="D8" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>4</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="C9" t="s">
         <v>183</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>184</v>
-      </c>
-      <c r="D9" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>5</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="C10" t="s">
+        <v>183</v>
+      </c>
+      <c r="D10" t="s">
         <v>186</v>
-      </c>
-      <c r="C10" t="s">
-        <v>184</v>
-      </c>
-      <c r="D10" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>188</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>189</v>
+      </c>
+      <c r="B14" t="s">
         <v>190</v>
-      </c>
-      <c r="B14" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>191</v>
+      </c>
+      <c r="B15" t="s">
         <v>192</v>
-      </c>
-      <c r="B15" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>193</v>
+      </c>
+      <c r="B16" t="s">
         <v>194</v>
-      </c>
-      <c r="B16" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="B17" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B18" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
   </sheetData>

</xml_diff>